<commit_message>
feat(dashboard): indicators and SLA page, decisions page, auto refresh, suggestions and traceability matrix
Add /indicadores with the eight calculable indicators grouped by audience,
plain-language insights derived from the rows, proposed SLA sheets marked
"a validar" and coverage first; restore the decisions list as /decisiones
with the most actionable insights. Replace the manual refresh button with
GET /api/v1/status polling that reloads only when the registry version
changes, plus an optional in-process sync scheduler (SYNC_INTERVAL_SECONDS)
guarded by the cross-process lock. Add suggestion and conflict sections,
paginated operations and the resolve action, the RF/RNF traceability
matrix exported with the other matrices, and a demo script in the README.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XY7P4gaUbUwedJunfzn1iZ
</commit_message>
<xml_diff>
--- a/output/matrices/matrices-econ.xlsx
+++ b/output/matrices/matrices-econ.xlsx
@@ -23,6 +23,7 @@
     <sheet name="Estados separados" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Evidencia de retorno" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="RACI propuesta" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Trazabilidad requisitos" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3135,6 +3136,660 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Requisito</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Qué exige el brief</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Evidencia en el repo (archivo o ruta exacta)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Dónde lo ve el jurado (URL de la app o documento)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Brecha y acción</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RF-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inventario de cualquier campo o término nuevo generado a partir del diccionario y dataset sandbox de Prisma y Startrack: nombre de campo, tipo de dato y ejemplo de valor.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>docs/diccionario-modelo-econ.md, generado por scripts/docs/generar_diccionario.py desde apps/api/app/models/hub.py, operations.py, workflow.py, graph.py, indicators.py y suggestions.py (nombre o JSONPath, tipo JSON, obligatorio, ejemplo con clase de evidencia, significado, procedencia); --check en scripts/check.sh y .github/workflows/ci.yml. Nombres equivalentes en el glosario de docs/equivalencias-prisma-startrack.md (output/matrices/glosario-sinonimos.csv, 36 conceptos).</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Documento docs/diccionario-modelo-econ.md; Swagger /docs (esquemas HubResponse, GraphProjection, IndicatorsReport, AssignmentSuggestion con descripción por campo); output/matrices/glosario-sinonimos.csv.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>El inventario cubre los modelos propios y sus derivaciones, no los DTO de los proveedores ni las 51 definiciones del kit (esas se cotejan en RF-02). Acción: regenerar con generar_diccionario.py tras cada cambio de modelo; CI falla si no coincide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RF-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Matriz de mapeo que conecte cada campo relevante de una plataforma con su equivalente en la otra, marcando explícitamente los campos sin equivalente directo.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>docs/equivalencias-prisma-startrack.md: clasificaciones directa, transformada, manual, sin equivalente y no soportada; formulario de tarea en cinco secciones; otros campos API del Job; inventario Prisma que no viaja; identidad y cardinalidad; inconsistencias del kit. Exportada a 16 CSV y output/matrices/matrices-econ.xlsx (manifiesto con SHA-256). Traza campo a campo en apps/api/app/services/integration_trace.py (field_map, tratamiento Conservado, Transformado, Manual o Sin equivalente) con pruebas en apps/api/tests/test_integration_trace.py.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>/integracion?mode=fixture (bloque «Mapeo campo a campo»); GET /api/v1/integration/{request_id} (field_map); output/matrices/formulario-tarea-completo.csv y otros-campos-api-tarea.csv; dossier output/pdf/ECON-entregables-visuales.pdf.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>parcial</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Falta el cotejo fila a fila de las 51 definiciones del diccionario del kit (12 Prisma, 39 Startrack) contra la matriz, y las correspondencias proyecto a geocerca, máquina a vehículo y operador a usuario no están validadas en la cuenta (la clave API de Startrack respondió 403). Acción: tabla de cotejo por fila del kit incluida en la exportación y validación autenticada; no inventar correspondencias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RF-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Matriz de responsabilidades que defina, para al menos tres roles funcionales, quién es Responsable, quién Aprueba, a quién se Consulta y a quién se Informa sobre el estado de un equipo (formato RACI recomendable).</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RACI de nueve decisiones en docs/equivalencias-prisma-startrack.md (sección «Responsabilidades propuestas para confirmar»: Gerencia de Proyecto, Logística y Equipo, Mantenimiento, Operador, Control de Costos, Soporte de integración, Responsable receptor) exportada a output/matrices/raci-propuesta.csv. Implementada como roles de sesión en apps/api/app/core/auth.py (admin, logistica, gerencia_proyecto, mantenimiento, control_costos, lectura; permisos read, manage_transfers, declare_reception, manage_users; docs/adr/0005-session-auth-and-roles.md) y actor registrado en operation_events.actor_* y en la recepción declared_by_* (migración 0004_guards, apps/api/migrations/versions/0004_movement_guards_actors_and_indexes.py).</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>/administracion (solo admin: alta de usuarios por rol); iniciar sesión con un usuario lectura y abrir /operaciones (sin acciones de gestión); /operaciones/{id} (actor de cada transición); output/matrices/raci-propuesta.csv; dossier PDF, páginas 2 a 4.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>La RACI es una propuesta pendiente de validación por las tres gerencias; el rol de sesión aplica permisos y registra quién actuó, no acredita esa aprobación. Acción: validar con ECON y fijar la denominación («Logística y Equipo» frente a «Maquinaria y Equipo» del organigrama).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RF-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>El prototipo debe permitir consultar el estado y la ubicación de al menos un equipo de forma unificada, combinando datos de ambas plataformas.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>/maquinaria/{id} en apps/api/app/dashboard/views.py (equipment_detail) con evidence_views.py (source_comparison, location_facts, maintenance_facts): estado administrativo y mantenimiento de Prisma, tarea y visita de Startrack conservadas en el registro, recepción declarada y ubicación fechada o «no verificable». GET /api/v1/hub (equipment[].transfers, location, provenance) y GET /api/v1/graph (gaps.machine_location, coverage). Pruebas: apps/api/tests/test_evidence_views.py, test_graph.py, test_hub_evidence_concordance.py.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>/maquinaria/{id}?mode=fixture (por ejemplo CF-03, nexus:equipment:66faacde-728c-4378-8b46-dbfb38254e03); grafo de portada /?mode=fixture seleccionando PROY-014; GET /api/v1/graph?mode=fixture.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>parcial</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>La vista combina ambas fuentes, pero ningún registro suministrado tiene evidencia de las dos: la muestra no trae tareas, visitas GPS ni recepciones y el acceso API de Startrack de la cuenta no está validado (403). El jurado ve hechos de Prisma y faltantes explícitos, no una ubicación observada. Acción: cadena live verificada (PROY-006) con tarea y visita reales, conservando IDs; no inventar registros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RF-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>El prototipo debe reflejar visualmente al menos un caso donde el estado del equipo difiere entre Prisma y Startrack, y cómo se resuelve.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Regla «OCUPADA en Prisma y tarea completada en Startrack coexisten» en apps/api/app/dashboard/evidence_views.py (interpretation_section) con pruebas en apps/api/tests/test_evidence_views.py; tensión obsolete_with_approved_request en apps/api/app/services/graph.py; estados por objeto en docs/equivalencias-prisma-startrack.md (sección «Fechas, unidades y estados separados», output/matrices/estados-separados.csv); diagrama 6 docs/assets/entregables/diagrama-estados.svg.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>/maquinaria/{id}?mode=fixture de CF-03 (OBSOLETA en Prisma con solicitud APROBADA: se muestra como tensión, no se «corrige»); GET /api/v1/graph?mode=fixture (tensions); docs/entregables-visuales.md, diagrama 6.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>parcial</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Con la muestra el caso compara solo hechos de Prisma; la regla Ocupada y Completada se ejercita con casos aislados de prueba, no con datos servidos. Acción: el mismo caso live de RF-04; en la demo decirlo así y no introducir una tarea inventada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RF-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Documentar al menos un indicador operativo que la integración haría visible por primera vez, por ejemplo tiempo de equipo fuera de geocerca sin justificación.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Definición única de «tiempo fuera de geocerca sin justificación» en docs/entregables-visuales.md (sección RF-06: unidad, cálculo, datos necesarios, decisión, resultado no evaluable). Ocho indicadores calculables por fila en apps/api/app/services/indicators.py (approval_time, open_request_age, approved_with_unit_without_sent_task, occupied_without_project, assignment_ended, completed_task_without_receipt, active_failure_registered, evidence_age) con fichas y SLA propuestos S1–S6 en docs/indicadores-calculables.md; pruebas en apps/api/tests/test_indicators.py.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>/indicadores?mode=fixture («Indicadores y SLA»: fichas por fila con estado evaluable, parcial o no evaluable, motivo y el SLA propuesto al lado); GET /api/v1/indicators?mode=fixture; dossier PDF, ficha RF-06 (páginas 14 a 16).</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>RF-06 no es calculable con la muestra (resultado no evaluable, no cero); los indicadores publicados describen filas de la lectura acotada, no la flota, y los umbrales de SLA están «a validar con ECON». Acción: no presentar promedios ni porcentajes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RNF-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Toda exploración y prueba exclusivamente sobre el entorno sandbox y los datasets sintéticos provistos por Grupo ECON.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Muestras con hash del documento en apps/api/app/integrations/data/sandbox_samples.json; ALLOW_LIVE_READS, ALLOW_LIVE_WRITES y AUTO_QUEUE_TRANSFERS en false por defecto (apps/api/app/core/config.py); conectores con origen fijo https://econ-key.maic.ai y https://staging.gps.gt/api (apps/api/app/integrations/nexus.py, startrack.py, http.py); evidence_kind provided_sample, live_read o test_case en apps/api/app/models/hub.py; pruebas apps/api/tests/test_security.py, test_nexus.py, test_startrack.py.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>/fuentes?mode=fixture (procedencia, alcance y estado de cada fuente); cada ficha lleva «Datos sintéticos».</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ninguna. Mantener la distinción fixture, live y caso de prueba en cada captura, cifra y demostración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RNF-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>La matriz de mapeo y la de responsabilidades en formato legible y reutilizable (hoja de cálculo o tabla estructurada), no solo texto libre.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>scripts/docs/exportar_matrices.py copia las tablas Markdown de docs/equivalencias-prisma-startrack.md y de esta matriz a output/matrices/*.csv (17 CSV UTF-8 con cabecera) y output/matrices/matrices-econ.xlsx (openpyxl 3.1.5, una hoja por tabla), con manifest.json y MANIFEST.md (SHA-256 del origen y de cada archivo); --check en scripts/check.sh y en CI.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>output/matrices/MANIFEST.md; abrir matrices-econ.xlsx; guía en README.md («Cómo revisar las matrices»).</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>El PDF output/pdf/ECON-diccionario-mapeo-y-manual-integracion.pdf (34 páginas, 12/09/2026) no tiene generador y no se regenera; el formato reutilizable vigente es Markdown más CSV/XLSX. Acción: regenerar tras cada edición (CI lo exige).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RNF-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Prototipo como dashboard, aplicación web o modelo de datos con interfaz mínima; navegable por el jurado.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Aplicación Dash y FastAPI en un proceso (apps/api/app/main.py); páginas en la tabla PAGES de apps/api/app/dashboard/views.py; accesibilidad por teclado en docs/frontend-architecture.md (sección «Accesibilidad»); capturas a 1280 y 390 px en docs/screenshots/2026-09-13-*.png; pruebas de callbacks y navegación en apps/api/tests/test_dashboard.py, test_workflow_ui.py y test_auth_ui.py.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8050/ tras /login; guion de diez pasos en README.md («Guion de demo para el jurado»).</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Navegabilidad y completitud de datos son dimensiones distintas: los faltantes de RF-04 y RF-05 siguen visibles. Acción: ensayar el guion sobre la entrega final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RNF-04</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Repositorio o carpeta de entrega con README que explique cómo revisar el prototipo y las matrices.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>README.md (Inicio, Recorrido, Guion de demo para el jurado, Cómo revisar las matrices, Sesión y roles, Verificar y desplegar), docs/README.md (índice) y apps/api/README.md; enlaces relativos comprobados.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>README.md.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Mantener los enlaces y los encabezados cuando cambien los documentos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>§9 Matriz de mapeo de campos</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Hoja de cálculo o tabla estructurada, incluidos los casos sin equivalente directo; medio: reporte en PDF.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Markdown y CSV/XLSX de RF-02 y RNF-02; el dossier output/pdf/ECON-entregables-visuales.pdf (16 páginas, 13/09/2026, output/pdf/MANIFEST.md) incluye RACI y diagramas, no la matriz completa; el PDF de 34 páginas del 12/09/2026 contiene una versión anterior sin generador.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>output/matrices/MANIFEST.md; output/pdf/MANIFEST.md.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>parcial</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>No existe un PDF vigente de la matriz completa. Acción: añadir a scripts/docs/generar_dossier.py un PDF de la matriz desde el Markdown, o entregar XLSX más Markdown declarándolo en la presentación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>§9 Matriz de responsabilidades</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tabla de roles frente a la plataforma integrada, al menos las tres gerencias involucradas; medio: PDF.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>RACI de RF-03: output/matrices/raci-propuesta.csv, páginas 2 a 4 del dossier PDF (RACI leída del Markdown por scripts/docs/generar_dossier.py), roles de sesión implementados.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Dossier PDF, páginas 2 a 4; raci-propuesta.csv; /administracion.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Rótulo de propuesta hasta la validación empresarial; las tres gerencias deben seguir visibles al resumirla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>§9 Prototipo o mockup navegable</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Al menos una consulta unificada; enlace o repositorio con instrucciones; el jurado elige un equipo o partida del sandbox y observa estado, ubicación y discrepancias.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Aplicación de RNF-03; scripts/dev.sh, docs/desarrollo.md; guion en README.md; en live (solo si el servidor lo habilita con credenciales) cualquier unidad o solicitud leída de Prisma se consulta por su ID.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>/maquinaria?mode=fixture (el jurado elige entre CF-01, CF-02, CF-03, EXC-01 y EXC-02) y su detalle; /solicitudes?mode=fixture.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>parcial</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>La consulta unificada con ambas plataformas depende de RF-04: con la muestra el jurado ve Prisma y faltantes explícitos; con live la lectura de Startrack sigue sin validar. Acción: cadena live verificada o declararlo en la demo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>§9 Diagrama de arquitectura</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Componentes, flujo de datos entre Prisma, Startrack y el prototipo, y dónde vive cada estado; medio: PDF.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Diagrama 3 (docs/assets/entregables/diagrama-actual.svg y .png) y diagrama 6 «dónde vive cada estado» (diagrama-estados.svg y .png), generados por scripts/docs/generar_dossier.py y registrados en docs/assets/entregables/manifest.json; texto y mermaid en docs/entregables-visuales.md y docs/solucion-integracion.md (sección «Arquitectura implementada»).</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>docs/entregables-visuales.md (diagramas 3 y 6); dossier PDF, páginas 8 a 13.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Los diagramas 4 y 5 son propuestas (sincronización y escala) y así se rotulan. Acción: mantener la separación implementado y propuesto en la presentación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>§9 Documento de decisiones técnicas</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Máximo dos páginas: qué se mapeó, qué se dejó fuera de alcance y por qué; medio: PDF.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>docs/decisiones-tecnicas.md y output/pdf/ECON-decisiones-tecnicas.pdf (2 páginas, 13/09/2026, SHA-256 en output/pdf/MANIFEST.md); scripts/docs/generar_dossier.py falla si supera dos páginas.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>output/pdf/ECON-decisiones-tecnicas.pdf; docs/decisiones-tecnicas.md.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Regenerar el PDF cuando cambie el Markdown y registrar el hash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>§9 Presentación final</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Máximo diez diapositivas: problema, solución, arquitectura, matrices y valor para Grupo ECON, con bloque de reflexión de aprendizaje; presentación en vivo.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>No existe en el repositorio. Insumos disponibles: dossier PDF (páginas 1 a 4: requisitos y RACI; 8 a 13: diagramas; 14 a 16: casos, RF-06 y recorrido) y guion de demo del README.md.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Acción: producir el archivo, contar diapositivas, incluir la reflexión real del equipo y mantener separadas capacidades implementadas y propuestas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>§6 Arquitectura de integración vía API (obligatorio)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Propuesta de arquitectura de integración entre ambas plataformas, más allá del mockup, con manejo de errores y sincronización de estados.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Estados de envío draft, blocked, queued, sending, sent, unknown y failed con conciliación sin reenviar y cierre explícito (POST /api/v1/operations/{id}/resolve) en apps/api/app/services/workflow.py y ledger.py; cola transaccional, exclusividad en vuelo por máquina, job_id único y operation_events append-only (migración 0004_guards; pruebas PostgreSQL apps/api/tests/test_postgres_*.py ejecutadas en CI); docs/solucion-integracion.md (secciones «Estados de envío y evidencia independiente» y «Tiempos del traslado»), docs/adr/0004-persistent-transfer-workflow.md, docs/adr/0006-postgresql-unica-infraestructura-de-estado.md; propuesta de sincronización y discrepancias en docs/sincronizacion-y-discrepancias.md.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>/operaciones/{id}?mode=fixture (estados, eventos y actor); /integracion?mode=fixture (payload preparado y respuesta esperada); Swagger /docs (POST /api/v1/operations/{id}/resolve, GET /api/v1/status).</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>La creación autenticada de tareas en la cuenta Startrack sigue sin validar y la detección de cambios de Prisma posteriores al envío es una señal del grafo (movement_source_changed), no una incidencia durable. Acción: validar credenciales y contrato; mantener la sincronización propuesta rotulada como tal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>§6 Panel de indicadores (deseable)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Panel que aborde al menos un síntoma identificado por ECON: tiempos muertos, baja trazabilidad o ausencia de indicadores unificados.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Página /indicadores («Indicadores y SLA», apps/api/app/dashboard/indicator_views.py) sobre GET /api/v1/indicators (apps/api/app/api/indicators.py, apps/api/app/services/indicators.py): ocho fichas agrupadas por área con lectura en lenguaje llano, filas, cobertura y SLA propuesto al lado; página /decisiones (views.py::decisions) con un asunto por solicitud, las tres lecturas más accionables de los indicadores, período de uso solicitado y distribución por estado (decision_priorities.py, decision_analytics.py); fichas y SLA en docs/indicadores-calculables.md; pruebas apps/api/tests/test_indicator_views.py y test_decision_priorities.py.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>/indicadores?mode=fixture; /decisiones?mode=fixture; GET /api/v1/indicators?mode=fixture.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Con la muestra la mayoría de las fichas queda «no evaluable» con motivo (sin corte, sin tareas) y ninguna publica promedios: el panel muestra cobertura, no desempeño. Acción: en live completar el registro antes de leerlo como serie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>§6 Escalabilidad y portal futuro (deseable)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Propuesta de cómo el mismo modelo podría extenderse a mayor escala, como un portal con visibilidad de tiempos de logística y disponibilidad de equipo.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Propuesta en docs/sincronizacion-y-discrepancias.md (sección «Escala a miles de vehículos (propuesta)»), diagrama 5 docs/assets/entregables/diagrama-escala.svg, extrapolación de retención y volumen en docs/database.md, y límites en docs/adr/0006-postgresql-unica-infraestructura-de-estado.md.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>docs/entregables-visuales.md (diagrama 5); dossier PDF, páginas 8 a 13.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>cumple</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Es una propuesta sin capacidad demostrada: faltan mediciones de carga, latencia y recuperación. Acción: presentarla como propuesta, no como despliegue.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(frontend): integrate redesigned Python Dash UI and align documentation
- Replace experimental Vite SPA with redesigned Python Dash interface (Dash Mantine, AG Grid, Plotly)
- Add KPI board (kpi_views.py), coverage analytics, and inventory analytics modules
- Add modular per-area stylesheets (z-kpi, z-flow, z-pages, z-shell, z-auth) and local fonts
- Add jury presentation pitch script (pitch.md), Q&A defense guide, and API contracts
- Optimize workflow polling cut and exclusiveness timeout in HTTP connector
- Align architectural documentation, README, and official deliverables
</commit_message>
<xml_diff>
--- a/output/matrices/matrices-econ.xlsx
+++ b/output/matrices/matrices-econ.xlsx
@@ -3291,7 +3291,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>/maquinaria/{id}?mode=fixture (por ejemplo CF-03, nexus:equipment:66faacde-728c-4378-8b46-dbfb38254e03); grafo de portada /?mode=fixture seleccionando PROY-014; GET /api/v1/graph?mode=fixture.</t>
+          <t>/maquinaria/{id}?mode=fixture (por ejemplo CF-03, nexus:equipment:66faacde-728c-4378-8b46-dbfb38254e03); la portada /?mode=fixture (asunto «Revisar la asignación» de esa unidad); GET /api/v1/graph?mode=fixture.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>/indicadores?mode=fixture («Indicadores y SLA»: fichas por fila con estado evaluable, parcial o no evaluable, motivo y el SLA propuesto al lado); GET /api/v1/indicators?mode=fixture; dossier PDF, ficha RF-06 (páginas 14 a 16).</t>
+          <t>/indicadores?mode=fixture: el «Tablero de indicadores» (trece cifras agrupadas por Logística, Proyectos, Mantenimiento e Información, cada una con su población y su cobertura, o con el motivo publicado cuando no hay población contable) y, debajo, una pestaña por pregunta con las filas y su estado (evaluable, parcial o no evaluable con motivo) más la pestaña «SLA propuestos» con los umbrales «a validar con ECON»; GET /api/v1/indicators?mode=fixture; dossier PDF, ficha RF-06 (páginas 14 a 16).</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Página /indicadores («Indicadores y SLA», apps/api/app/dashboard/indicator_views.py) sobre GET /api/v1/indicators (apps/api/app/api/indicators.py, apps/api/app/services/indicators.py): ocho fichas agrupadas por área con lectura en lenguaje llano, filas, cobertura y SLA propuesto al lado; página /decisiones (views.py::decisions) con un asunto por solicitud, las tres lecturas más accionables de los indicadores, período de uso solicitado y distribución por estado (decision_priorities.py, decision_analytics.py); fichas y SLA en docs/indicadores-calculables.md; pruebas apps/api/tests/test_indicator_views.py y test_decision_priorities.py.</t>
+          <t>Página /indicadores (apps/api/app/dashboard/indicator_views.py con kpi_views.py) sobre GET /api/v1/indicators (apps/api/app/api/indicators.py, apps/api/app/services/indicators.py): tablero de trece cifras agrupadas por el área que decide —Logística, Proyectos, Mantenimiento e Información—, cada una con su población, su cobertura y el enlace a las filas que la sustentan, y debajo una pestaña por pregunta (lectura en lenguaje llano, filas y cobertura) más la pestaña «SLA propuestos»; reglas del tablero en docs/kpis-tablero.md. Página /decisiones (views.py::decisions, la misma que la portada /) con «Qué pasa · Agenda de uso y asignación» sobre el período de uso solicitado y «Qué hago · Acciones por solicitud» con un asunto por solicitud, su hecho observado y su siguiente paso (decision_priorities.py, decision_analytics.py); el conteo por estado de solicitud queda como tabla en el desplegable «Datos de la agenda». Fichas y SLA en docs/indicadores-calculables.md; pruebas apps/api/tests/test_indicator_views.py y test_decision_priorities.py.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Con la muestra la mayoría de las fichas queda «no evaluable» con motivo (sin corte, sin tareas) y ninguna publica promedios: el panel muestra cobertura, no desempeño. Acción: en live completar el registro antes de leerlo como serie.</t>
+          <t>Con la muestra la mayoría de las cifras y fichas queda «no evaluable» con motivo (sin corte, sin tareas) y ninguna publica promedios: el panel muestra cobertura, no desempeño. Corrección del 13/09/2026: esta celda citaba «las tres lecturas más accionables de los indicadores» y una «distribución por estado» en /decisiones; ninguna de las dos existe hoy —indicator_insights dejó de montarse en esa página y el gráfico de estados se retiró de la portada—, y la capacidad que sostiene el veredicto es ahora el tablero de /indicadores. Pendiente: indicator_insights y top_insights siguen en indicator_views.py sin uso en ninguna página. Acción: en live completar el registro antes de leerlo como serie.</t>
         </is>
       </c>
     </row>

</xml_diff>